<commit_message>
add vanilla OXL time functions ported to AXL + update test sheet
modified:   sheets/axl_demo_test.xlsx
modified:   test/CMakeLists.txt
modified:   test/axl_demo.cpp
</commit_message>
<xml_diff>
--- a/sheets/axl_demo_test.xlsx
+++ b/sheets/axl_demo_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Derek\START\prog_proj\OdinAnalytics\sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F266F281-7D71-4528-A1F4-0A1C9FF3CA88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA76375-0927-411F-B650-6E8B80CD21E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{CC038B3D-5DA1-43AC-BE17-600265123F86}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
   <si>
     <t xml:space="preserve">apple </t>
   </si>
@@ -148,7 +148,58 @@
     <t>Date Functions</t>
   </si>
   <si>
-    <t>(TBD)</t>
+    <t>Base_Date</t>
+  </si>
+  <si>
+    <t>Tenor</t>
+  </si>
+  <si>
+    <t>Calendar</t>
+  </si>
+  <si>
+    <t>Adjustment_Rule</t>
+  </si>
+  <si>
+    <t>8M</t>
+  </si>
+  <si>
+    <t>Following</t>
+  </si>
+  <si>
+    <t>NYB</t>
+  </si>
+  <si>
+    <t>NYB;LNB</t>
+  </si>
+  <si>
+    <t>=AxIsBusinessDay(P9,Q9)</t>
+  </si>
+  <si>
+    <t>=AxIsBusinessDay(P10,Q10)</t>
+  </si>
+  <si>
+    <t>=AxIsHoliday(P9,Q9)</t>
+  </si>
+  <si>
+    <t>=AxIsHoliday(P10,Q10)</t>
+  </si>
+  <si>
+    <t>ACT/ACT</t>
+  </si>
+  <si>
+    <t>30/360</t>
+  </si>
+  <si>
+    <t>=AxDayCount(P9,P10,P12)</t>
+  </si>
+  <si>
+    <t>=AxDayCount(P9,P10,Q12)</t>
+  </si>
+  <si>
+    <t>=AxYearFraction(P9,P10,P12)</t>
+  </si>
+  <si>
+    <t>=AxYearFraction(P9,P10,Q12)</t>
   </si>
 </sst>
 </file>
@@ -324,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -342,6 +393,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -695,7 +753,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C818C1D-2C17-41AA-9577-0406209DFD12}">
-  <dimension ref="B1:P59"/>
+  <dimension ref="B2:Q59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="4" width="9.140625" customWidth="1"/>
@@ -704,39 +762,34 @@
     <col min="8" max="8" width="9.140625" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="13.28515625" customWidth="1"/>
-    <col min="13" max="14" width="9.140625" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.85546875" customWidth="1"/>
+    <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="I1" t="str" cm="1">
-        <f t="array" ref="I1">_xll.AxDictionary(I9:K9,I10:K10)</f>
-        <v>Dictionary_Inventory_$0$8:6</v>
-      </c>
-    </row>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>14</v>
       </c>
       <c r="G3" s="1"/>
     </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="15"/>
       <c r="D5" s="16"/>
-      <c r="M5" s="14" t="s">
+      <c r="M5" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="N5" s="16"/>
-    </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="N5" s="12"/>
+    </row>
+    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
         <v>16</v>
       </c>
@@ -746,11 +799,14 @@
       <c r="I7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="M7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="P7" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>1</v>
       </c>
@@ -767,7 +823,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>0</v>
       </c>
@@ -792,8 +848,20 @@
       <c r="K9" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N9" s="17">
+        <v>45163</v>
+      </c>
+      <c r="P9" s="18">
+        <v>46016</v>
+      </c>
+      <c r="Q9" s="16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>15</v>
       </c>
@@ -818,8 +886,28 @@
       <c r="K10" s="8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="N10" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="P10" s="18">
+        <v>46049</v>
+      </c>
+      <c r="Q10" s="16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="M11" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
         <v>17</v>
       </c>
@@ -829,22 +917,34 @@
       <c r="I12" s="10" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="N12" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="P12" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q12" s="16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" t="str" cm="1">
         <f t="array" ref="B13">_xll.AxArray(B8:C10)</f>
-        <v>Array_Inventory_$12$1:2</v>
+        <v>Array_Inventory_$12$1:1</v>
       </c>
       <c r="E13" t="str" cm="1">
         <f t="array" ref="E13">_xll.AxDictionary($E$8:$E$10,F8:F10)</f>
-        <v>Dictionary_Inventory_$12$4:2</v>
+        <v>Dictionary_Inventory_$12$4:1</v>
       </c>
       <c r="I13" t="str" cm="1">
         <f t="array" ref="I13">_xll.AxDictionary(I9:K9,I10:K10)</f>
-        <v>Dictionary_Inventory_$12$8:0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.25">
+        <v>Dictionary_Inventory_$12$8:3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>18</v>
       </c>
@@ -854,8 +954,11 @@
       <c r="I15" s="10" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="P15" s="10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B16" t="str" cm="1">
         <f t="array" ref="B16:C18">_xll.AxDisplay(B13)</f>
         <v>jack fruit</v>
@@ -877,8 +980,12 @@
       <c r="J16" t="str">
         <v>Royal Oak: 50</v>
       </c>
-    </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="P16" t="b" cm="1">
+        <f t="array" ref="P16">_xll.AxIsBusinessDay(P9,Q9)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <v xml:space="preserve">apple </v>
       </c>
@@ -898,7 +1005,7 @@
         <v>Polaris:6</v>
       </c>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <v>banana</v>
       </c>
@@ -917,8 +1024,17 @@
       <c r="J18" t="str">
         <v>DayTona:60</v>
       </c>
-    </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="P18" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P19" t="b" cm="1">
+        <f t="array" ref="P19">_xll.AxIsBusinessDay(P10,Q10)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="10" t="s">
         <v>19</v>
       </c>
@@ -926,17 +1042,26 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" t="str" cm="1">
         <f t="array" ref="B21">_xll.AxArray(B16:C16)</f>
-        <v>Array_Inventory_$20$1:2</v>
+        <v>Array_Inventory_$20$1:1</v>
       </c>
       <c r="E21" t="str" cm="1">
         <f t="array" ref="E21">_xll.AxDictionary($E$8:$E$10,G8:G10)</f>
-        <v>Dictionary_Inventory_$20$4:2</v>
-      </c>
-    </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+        <v>Dictionary_Inventory_$20$4:1</v>
+      </c>
+      <c r="P21" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P22" t="b" cm="1">
+        <f t="array" ref="P22">_xll.AxIsHoliday(P9,Q9)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="10" t="s">
         <v>20</v>
       </c>
@@ -944,7 +1069,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" t="str" cm="1">
         <f t="array" ref="B24:C24">_xll.AxDisplay(B21)</f>
         <v>jack fruit</v>
@@ -959,16 +1084,23 @@
       <c r="F24" t="str">
         <v>Royal Oak:20</v>
       </c>
-    </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="P24" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="E25" t="str">
         <v>JLC</v>
       </c>
       <c r="F25" t="str">
         <v>Reverso:250</v>
       </c>
-    </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="P25" t="b" cm="1">
+        <f t="array" ref="P25">_xll.AxIsHoliday(P10,Q10)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="E26" t="str">
         <v>Rolex</v>
       </c>
@@ -976,11 +1108,53 @@
         <v>Oyster Perpetual:15</v>
       </c>
     </row>
-    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P27" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P28" cm="1">
+        <f t="array" ref="P28">_xll.AxDayCount(P9,P10,P12)</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P30" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="P31" cm="1">
+        <f t="array" ref="P31">_xll.AxDayCount(P9,P10,Q12)</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="M32" s="2"/>
+    </row>
+    <row r="33" spans="8:16" x14ac:dyDescent="0.25">
+      <c r="P33" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="8:16" x14ac:dyDescent="0.25">
+      <c r="P34" cm="1">
+        <f t="array" ref="P34">_xll.AxYearFraction(P9,P10,P12)</f>
+        <v>9.0410958904109592E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="8:16" x14ac:dyDescent="0.25">
+      <c r="P36" s="10" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="37" spans="8:16" x14ac:dyDescent="0.25">
       <c r="H37" s="1"/>
+      <c r="P37" cm="1">
+        <f t="array" ref="P37">_xll.AxYearFraction(P9,P10,Q12)</f>
+        <v>8.8888888888888892E-2</v>
+      </c>
     </row>
     <row r="38" spans="8:16" x14ac:dyDescent="0.25">
       <c r="H38" s="1"/>

</xml_diff>

<commit_message>
add AxComputeDate() + update test sheet
modified:   sheets/axl_demo_test.xlsx
modified:   test/axl_demo.cpp
</commit_message>
<xml_diff>
--- a/sheets/axl_demo_test.xlsx
+++ b/sheets/axl_demo_test.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Derek\START\prog_proj\OdinAnalytics\sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EA76375-0927-411F-B650-6E8B80CD21E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE134A6E-AC09-4C36-A073-11499C2862CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{CC038B3D-5DA1-43AC-BE17-600265123F86}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{CC038B3D-5DA1-43AC-BE17-600265123F86}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Inventory" sheetId="2" r:id="rId2"/>
+    <sheet name="main" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
   <si>
     <t xml:space="preserve">apple </t>
   </si>
@@ -103,9 +102,6 @@
     <t>AXL Demo Test</t>
   </si>
   <si>
-    <t>This demonstrates OXL array and time functions using the Accel framework.</t>
-  </si>
-  <si>
     <t>banana</t>
   </si>
   <si>
@@ -200,6 +196,21 @@
   </si>
   <si>
     <t>=AxYearFraction(P9,P10,Q12)</t>
+  </si>
+  <si>
+    <t>=AxComputeDate(M9:N12)</t>
+  </si>
+  <si>
+    <t>=AxComputeDate(M9:M12,N9:N12)</t>
+  </si>
+  <si>
+    <t>This demonstrates OXL array and time functions exported using the Accel framework.</t>
+  </si>
+  <si>
+    <t>=AxDictionary(M9:M12,N9:N12)</t>
+  </si>
+  <si>
+    <t>=AxComputeDate(M22)</t>
   </si>
 </sst>
 </file>
@@ -375,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -393,6 +404,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -713,45 +727,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10DFABD2-AE01-4866-8EEF-6EB1F781458C}">
-  <dimension ref="B7:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="9" max="9" width="32.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.28515625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B7" t="str">
-        <f t="array" ref="B7:C9">_xll.oxlDisplay(Inventory!D25)</f>
-        <v>ERROR:Not an Excel String Type line check the input: xloper_converter.cpp line 244 LPXloperToStr()</v>
-      </c>
-      <c r="C7" t="str">
-        <v>ERROR:Not an Excel String Type line check the input: xloper_converter.cpp line 244 LPXloperToStr()</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B8" t="str">
-        <v>ERROR:Not an Excel String Type line check the input: xloper_converter.cpp line 244 LPXloperToStr()</v>
-      </c>
-      <c r="C8" t="str">
-        <v>ERROR:Not an Excel String Type line check the input: xloper_converter.cpp line 244 LPXloperToStr()</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B9" t="str">
-        <v>ERROR:Not an Excel String Type line check the input: xloper_converter.cpp line 244 LPXloperToStr()</v>
-      </c>
-      <c r="C9" t="str">
-        <v>ERROR:Not an Excel String Type line check the input: xloper_converter.cpp line 244 LPXloperToStr()</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C818C1D-2C17-41AA-9577-0406209DFD12}">
   <dimension ref="B2:Q59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -774,36 +749,36 @@
     </row>
     <row r="3" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="5" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="15"/>
       <c r="D5" s="16"/>
       <c r="M5" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N5" s="12"/>
     </row>
     <row r="7" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="2:17" x14ac:dyDescent="0.25">
@@ -849,21 +824,21 @@
         <v>4</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="N9" s="17">
+        <v>28</v>
+      </c>
+      <c r="N9" s="18">
         <v>45163</v>
       </c>
-      <c r="P9" s="18">
+      <c r="P9" s="19">
         <v>46016</v>
       </c>
       <c r="Q9" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C10" s="8">
         <v>120</v>
@@ -887,75 +862,78 @@
         <v>6</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="P10" s="18">
+        <v>32</v>
+      </c>
+      <c r="P10" s="19">
         <v>46049</v>
       </c>
       <c r="Q10" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="2:17" x14ac:dyDescent="0.25">
       <c r="M11" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="N12" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="P12" s="19" t="s">
+        <v>34</v>
+      </c>
+      <c r="P12" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q12" s="16" t="s">
         <v>41</v>
-      </c>
-      <c r="Q12" s="16" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="13" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B13" t="str" cm="1">
         <f t="array" ref="B13">_xll.AxArray(B8:C10)</f>
-        <v>Array_Inventory_$12$1:1</v>
+        <v>Array_main_$12$1:0</v>
       </c>
       <c r="E13" t="str" cm="1">
         <f t="array" ref="E13">_xll.AxDictionary($E$8:$E$10,F8:F10)</f>
-        <v>Dictionary_Inventory_$12$4:1</v>
+        <v>Dictionary_main_$12$4:0</v>
       </c>
       <c r="I13" t="str" cm="1">
         <f t="array" ref="I13">_xll.AxDictionary(I9:K9,I10:K10)</f>
-        <v>Dictionary_Inventory_$12$8:3</v>
+        <v>Dictionary_main_$12$8:0</v>
       </c>
     </row>
     <row r="15" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>46</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:17" x14ac:dyDescent="0.25">
@@ -980,6 +958,10 @@
       <c r="J16" t="str">
         <v>Royal Oak: 50</v>
       </c>
+      <c r="M16" s="17" cm="1">
+        <f t="array" ref="M16">_xll.AxComputeDate(M9:N12)</f>
+        <v>45407</v>
+      </c>
       <c r="P16" t="b" cm="1">
         <f t="array" ref="P16">_xll.AxIsBusinessDay(P9,Q9)</f>
         <v>0</v>
@@ -1024,11 +1006,18 @@
       <c r="J18" t="str">
         <v>DayTona:60</v>
       </c>
+      <c r="M18" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="P18" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="M19" s="17" cm="1">
+        <f t="array" ref="M19">_xll.AxComputeDate(M9:M12,N9:N12)</f>
+        <v>45407</v>
+      </c>
       <c r="P19" t="b" cm="1">
         <f t="array" ref="P19">_xll.AxIsBusinessDay(P10,Q10)</f>
         <v>1</v>
@@ -1036,26 +1025,33 @@
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" t="str" cm="1">
         <f t="array" ref="B21">_xll.AxArray(B16:C16)</f>
-        <v>Array_Inventory_$20$1:1</v>
+        <v>Array_main_$20$1:0</v>
       </c>
       <c r="E21" t="str" cm="1">
         <f t="array" ref="E21">_xll.AxDictionary($E$8:$E$10,G8:G10)</f>
-        <v>Dictionary_Inventory_$20$4:1</v>
+        <v>Dictionary_main_$20$4:0</v>
+      </c>
+      <c r="M21" s="10" t="s">
+        <v>49</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="M22" t="str" cm="1">
+        <f t="array" ref="M22">_xll.AxDictionary(M9:M12,N9:N12)</f>
+        <v>Dictionary_main_$21$12:0</v>
+      </c>
       <c r="P22" t="b" cm="1">
         <f t="array" ref="P22">_xll.AxIsHoliday(P9,Q9)</f>
         <v>1</v>
@@ -1063,10 +1059,10 @@
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
@@ -1084,8 +1080,11 @@
       <c r="F24" t="str">
         <v>Royal Oak:20</v>
       </c>
+      <c r="M24" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="P24" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
@@ -1095,6 +1094,10 @@
       <c r="F25" t="str">
         <v>Reverso:250</v>
       </c>
+      <c r="M25" s="17" cm="1">
+        <f t="array" ref="M25">_xll.AxComputeDate(M22)</f>
+        <v>45407</v>
+      </c>
       <c r="P25" t="b" cm="1">
         <f t="array" ref="P25">_xll.AxIsHoliday(P10,Q10)</f>
         <v>0</v>
@@ -1110,7 +1113,7 @@
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.25">
       <c r="P27" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
@@ -1121,7 +1124,7 @@
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="P30" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="2:16" x14ac:dyDescent="0.25">
@@ -1135,7 +1138,7 @@
     </row>
     <row r="33" spans="8:16" x14ac:dyDescent="0.25">
       <c r="P33" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" spans="8:16" x14ac:dyDescent="0.25">
@@ -1146,7 +1149,7 @@
     </row>
     <row r="36" spans="8:16" x14ac:dyDescent="0.25">
       <c r="P36" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="8:16" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
axl_demo_test.xlsx: update with AxAddBusinessDays()
</commit_message>
<xml_diff>
--- a/sheets/axl_demo_test.xlsx
+++ b/sheets/axl_demo_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Derek\START\prog_proj\OdinAnalytics\sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE134A6E-AC09-4C36-A073-11499C2862CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45D599A7-3E0C-4ED1-9B45-4BB285FFE53A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{CC038B3D-5DA1-43AC-BE17-600265123F86}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="63">
   <si>
     <t xml:space="preserve">apple </t>
   </si>
@@ -211,6 +211,42 @@
   </si>
   <si>
     <t>=AxComputeDate(M22)</t>
+  </si>
+  <si>
+    <t>=AxDisplay(M22)</t>
+  </si>
+  <si>
+    <t>Days</t>
+  </si>
+  <si>
+    <t>=AxAddBusinessDays(S8:T10)</t>
+  </si>
+  <si>
+    <t>=AxAddBusinessDays(S8:S10,T8:T10)</t>
+  </si>
+  <si>
+    <t>=AxDictionary(S8:S10,T8:T10)</t>
+  </si>
+  <si>
+    <t>=AxDisplay(S19)</t>
+  </si>
+  <si>
+    <t>=AxAddBusinessDays(S19)</t>
+  </si>
+  <si>
+    <t>=AxAddBusinessDays(U8:V10)</t>
+  </si>
+  <si>
+    <t>=AxAddBusinessDays(U8:U10,V8:V10)</t>
+  </si>
+  <si>
+    <t>=AxDictionary(U8:U10,V8:V10)</t>
+  </si>
+  <si>
+    <t>=AxDisplay(V19)</t>
+  </si>
+  <si>
+    <t>=AxAddBusinessDays(V19)</t>
   </si>
 </sst>
 </file>
@@ -386,7 +422,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -414,6 +450,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -728,7 +770,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C818C1D-2C17-41AA-9577-0406209DFD12}">
-  <dimension ref="B2:Q59"/>
+  <dimension ref="B2:W59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="4" width="9.140625" customWidth="1"/>
@@ -740,20 +782,24 @@
     <col min="13" max="13" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.85546875" customWidth="1"/>
     <col min="16" max="16" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>48</v>
       </c>
       <c r="G3" s="1"/>
     </row>
-    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" s="14" t="s">
         <v>20</v>
       </c>
@@ -764,7 +810,7 @@
       </c>
       <c r="N5" s="12"/>
     </row>
-    <row r="7" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" s="9" t="s">
         <v>15</v>
       </c>
@@ -780,8 +826,11 @@
       <c r="P7" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="8" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="S7" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" s="3" t="s">
         <v>1</v>
       </c>
@@ -797,8 +846,26 @@
       <c r="G8" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P8" s="19">
+        <v>46016</v>
+      </c>
+      <c r="Q8" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="T8" s="18">
+        <v>46336</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="V8" s="18">
+        <v>46344</v>
+      </c>
+    </row>
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>0</v>
       </c>
@@ -830,13 +897,25 @@
         <v>45163</v>
       </c>
       <c r="P9" s="19">
-        <v>46016</v>
+        <v>46049</v>
       </c>
       <c r="Q9" s="16" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="10" spans="2:17" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="S9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="T9" s="22">
+        <v>5</v>
+      </c>
+      <c r="U9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="V9" s="22">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>14</v>
       </c>
@@ -867,14 +946,26 @@
       <c r="N10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="P10" s="19">
-        <v>46049</v>
+      <c r="P10" s="20" t="s">
+        <v>40</v>
       </c>
       <c r="Q10" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="S10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T10" s="8" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="U10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="V10" s="8" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="M11" s="5" t="s">
         <v>31</v>
       </c>
@@ -882,7 +973,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
         <v>16</v>
       </c>
@@ -898,14 +989,14 @@
       <c r="N12" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="P12" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q12" s="16" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="P12" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="S12" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="str" cm="1">
         <f t="array" ref="B13">_xll.AxArray(B8:C10)</f>
         <v>Array_main_$12$1:0</v>
@@ -916,10 +1007,18 @@
       </c>
       <c r="I13" t="str" cm="1">
         <f t="array" ref="I13">_xll.AxDictionary(I9:K9,I10:K10)</f>
-        <v>Dictionary_main_$12$8:0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:17" x14ac:dyDescent="0.25">
+        <v>Dictionary_main_$12$8:2</v>
+      </c>
+      <c r="P13" t="b" cm="1">
+        <f t="array" ref="P13">_xll.AxIsBusinessDay(P8,Q8)</f>
+        <v>0</v>
+      </c>
+      <c r="S13" s="17" cm="1">
+        <f t="array" ref="S13">_xll.AxAddBusinessDays(S8:T10)</f>
+        <v>46344</v>
+      </c>
+    </row>
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" s="10" t="s">
         <v>17</v>
       </c>
@@ -933,10 +1032,13 @@
         <v>46</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="2:17" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="S15" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" t="str" cm="1">
         <f t="array" ref="B16:C18">_xll.AxDisplay(B13)</f>
         <v>jack fruit</v>
@@ -964,10 +1066,14 @@
       </c>
       <c r="P16" t="b" cm="1">
         <f t="array" ref="P16">_xll.AxIsBusinessDay(P9,Q9)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="S16" s="17" cm="1">
+        <f t="array" ref="S16">_xll.AxAddBusinessDays(S8:S10,T8:T10)</f>
+        <v>46344</v>
+      </c>
+    </row>
+    <row r="17" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <v xml:space="preserve">apple </v>
       </c>
@@ -987,7 +1093,7 @@
         <v>Polaris:6</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <v>banana</v>
       </c>
@@ -1010,20 +1116,34 @@
         <v>47</v>
       </c>
       <c r="P18" s="10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="S18" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="V18" s="10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
       <c r="M19" s="17" cm="1">
         <f t="array" ref="M19">_xll.AxComputeDate(M9:M12,N9:N12)</f>
         <v>45407</v>
       </c>
       <c r="P19" t="b" cm="1">
-        <f t="array" ref="P19">_xll.AxIsBusinessDay(P10,Q10)</f>
+        <f t="array" ref="P19">_xll.AxIsHoliday(P8,Q8)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="S19" t="str" cm="1">
+        <f t="array" ref="S19">_xll.AxDictionary(S8:S10,T8:T10)</f>
+        <v>Dictionary_main_$18$18:2</v>
+      </c>
+      <c r="V19" t="str" cm="1">
+        <f t="array" ref="V19">_xll.AxDictionary(U8:U10,V8:V10)</f>
+        <v>Dictionary_main_$17$21:0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B20" s="10" t="s">
         <v>18</v>
       </c>
@@ -1031,7 +1151,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B21" t="str" cm="1">
         <f t="array" ref="B21">_xll.AxArray(B16:C16)</f>
         <v>Array_main_$20$1:0</v>
@@ -1044,28 +1164,60 @@
         <v>49</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="S21" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="V21" s="10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="2:23" x14ac:dyDescent="0.25">
       <c r="M22" t="str" cm="1">
         <f t="array" ref="M22">_xll.AxDictionary(M9:M12,N9:N12)</f>
-        <v>Dictionary_main_$21$12:0</v>
+        <v>Dictionary_main_$21$12:1</v>
       </c>
       <c r="P22" t="b" cm="1">
         <f t="array" ref="P22">_xll.AxIsHoliday(P9,Q9)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="S22" t="str" cm="1">
+        <f t="array" ref="S22:T24">_xll.AxDisplay(S19)</f>
+        <v>Base_Date</v>
+      </c>
+      <c r="T22" s="17">
+        <v>46336</v>
+      </c>
+      <c r="V22" t="str" cm="1">
+        <f t="array" ref="V22:W24">_xll.AxDisplay(V19)</f>
+        <v>Base_Date</v>
+      </c>
+      <c r="W22" s="17">
+        <v>46344</v>
+      </c>
+    </row>
+    <row r="23" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B23" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="S23" t="str">
+        <v>Calendar</v>
+      </c>
+      <c r="T23" t="str">
+        <v>NYB</v>
+      </c>
+      <c r="V23" t="str">
+        <v>Calendar</v>
+      </c>
+      <c r="W23" t="str">
+        <v>NYB</v>
+      </c>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.25">
       <c r="B24" t="str" cm="1">
         <f t="array" ref="B24:C24">_xll.AxDisplay(B21)</f>
         <v>jack fruit</v>
@@ -1081,94 +1233,152 @@
         <v>Royal Oak:20</v>
       </c>
       <c r="M24" s="10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="P24" s="10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Days</v>
+      </c>
+      <c r="T24" s="21">
+        <v>5</v>
+      </c>
+      <c r="V24" t="str">
+        <v>Days</v>
+      </c>
+      <c r="W24" s="21">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="25" spans="2:23" x14ac:dyDescent="0.25">
       <c r="E25" t="str">
         <v>JLC</v>
       </c>
       <c r="F25" t="str">
         <v>Reverso:250</v>
       </c>
-      <c r="M25" s="17" cm="1">
-        <f t="array" ref="M25">_xll.AxComputeDate(M22)</f>
-        <v>45407</v>
-      </c>
-      <c r="P25" t="b" cm="1">
-        <f t="array" ref="P25">_xll.AxIsHoliday(P10,Q10)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="M25" t="str" cm="1">
+        <f t="array" ref="M25:N28">_xll.AxDisplay(M22)</f>
+        <v>Adjustment_Rule</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Following</v>
+      </c>
+      <c r="P25" cm="1">
+        <f t="array" ref="P25">_xll.AxDayCount(P8,P9,P10)</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="2:23" x14ac:dyDescent="0.25">
       <c r="E26" t="str">
         <v>Rolex</v>
       </c>
       <c r="F26" t="str">
         <v>Oyster Perpetual:15</v>
       </c>
-    </row>
-    <row r="27" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="M26" t="str">
+        <v>Base_Date</v>
+      </c>
+      <c r="N26">
+        <v>45163</v>
+      </c>
+    </row>
+    <row r="27" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="M27" t="str">
+        <v>Calendar</v>
+      </c>
+      <c r="N27" t="str">
+        <v>NYB</v>
+      </c>
       <c r="P27" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="S27" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="28" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="M28" t="str">
+        <v>Tenor</v>
+      </c>
+      <c r="N28" t="str">
+        <v>8M</v>
+      </c>
       <c r="P28" cm="1">
-        <f t="array" ref="P28">_xll.AxDayCount(P9,P10,P12)</f>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+        <f t="array" ref="P28">_xll.AxDayCount(P8,P9,Q10)</f>
+        <v>32</v>
+      </c>
+      <c r="S28" s="17" cm="1">
+        <f t="array" ref="S28">_xll.AxAddBusinessDays(S19)</f>
+        <v>46344</v>
+      </c>
+    </row>
+    <row r="30" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="M30" s="10" t="s">
+        <v>50</v>
+      </c>
       <c r="P30" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+      <c r="S30" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="31" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="M31" s="17" cm="1">
+        <f t="array" ref="M31">_xll.AxComputeDate(M22)</f>
+        <v>45407</v>
+      </c>
       <c r="P31" cm="1">
-        <f t="array" ref="P31">_xll.AxDayCount(P9,P10,Q12)</f>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="M32" s="2"/>
-    </row>
-    <row r="33" spans="8:16" x14ac:dyDescent="0.25">
+        <f t="array" ref="P31">_xll.AxYearFraction(P8,P9,P10)</f>
+        <v>9.0410958904109592E-2</v>
+      </c>
+      <c r="S31" s="17" cm="1">
+        <f t="array" ref="S31">_xll.AxAddBusinessDays(U8:V10)</f>
+        <v>46336</v>
+      </c>
+    </row>
+    <row r="33" spans="8:19" x14ac:dyDescent="0.25">
       <c r="P33" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="34" spans="8:16" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="S33" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" spans="8:19" x14ac:dyDescent="0.25">
       <c r="P34" cm="1">
-        <f t="array" ref="P34">_xll.AxYearFraction(P9,P10,P12)</f>
-        <v>9.0410958904109592E-2</v>
-      </c>
-    </row>
-    <row r="36" spans="8:16" x14ac:dyDescent="0.25">
-      <c r="P36" s="10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="37" spans="8:16" x14ac:dyDescent="0.25">
+        <f t="array" ref="P34">_xll.AxYearFraction(P8,P9,Q10)</f>
+        <v>8.8888888888888892E-2</v>
+      </c>
+      <c r="S34" s="17" cm="1">
+        <f t="array" ref="S34">_xll.AxAddBusinessDays(U8:U10,V8:V10)</f>
+        <v>46336</v>
+      </c>
+    </row>
+    <row r="36" spans="8:19" x14ac:dyDescent="0.25">
+      <c r="S36" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="37" spans="8:19" x14ac:dyDescent="0.25">
       <c r="H37" s="1"/>
-      <c r="P37" cm="1">
-        <f t="array" ref="P37">_xll.AxYearFraction(P9,P10,Q12)</f>
-        <v>8.8888888888888892E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="8:16" x14ac:dyDescent="0.25">
+      <c r="S37" s="17" cm="1">
+        <f t="array" ref="S37">_xll.AxAddBusinessDays(V19)</f>
+        <v>46336</v>
+      </c>
+    </row>
+    <row r="38" spans="8:19" x14ac:dyDescent="0.25">
       <c r="H38" s="1"/>
     </row>
-    <row r="39" spans="8:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="8:19" x14ac:dyDescent="0.25">
       <c r="H39" s="1"/>
     </row>
-    <row r="40" spans="8:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="8:19" x14ac:dyDescent="0.25">
       <c r="H40" s="1"/>
     </row>
-    <row r="48" spans="8:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="8:19" x14ac:dyDescent="0.25">
       <c r="N48" s="1"/>
       <c r="P48" s="1"/>
     </row>

</xml_diff>